<commit_message>
upgrade to dot net 8
</commit_message>
<xml_diff>
--- a/CS/SpreadsheetDocServerAPIPart2/Document.xlsx
+++ b/CS/SpreadsheetDocServerAPIPart2/Document.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27830"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D29DD6B-C22A-45DE-9DE8-B6C22F49408E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E6EDABE-0BE7-44FB-ADB8-EAC462D64D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,8 +21,8 @@
     <sheet name="Regional Sales" sheetId="25" state="hidden" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">SortSample!$A$2:$F$22</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="7">SortSample!$B$2:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">SortSample!$A$2:$D$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">SortSample!$B$2:$B$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="96">
   <si>
     <t>Price</t>
   </si>
@@ -153,12 +153,6 @@
     <t>Symbol</t>
   </si>
   <si>
-    <t>Population, thousand</t>
-  </si>
-  <si>
-    <t>GDP, USD mln</t>
-  </si>
-  <si>
     <t>Area, thousand hectares</t>
   </si>
   <si>
@@ -244,12 +238,6 @@
   </si>
   <si>
     <t>MEX</t>
-  </si>
-  <si>
-    <t>Russian Federation</t>
-  </si>
-  <si>
-    <t>RUS</t>
   </si>
   <si>
     <t>Saudi Arabia</t>
@@ -353,7 +341,7 @@
     <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     <numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(_)"/>
   </numFmts>
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -541,13 +529,6 @@
       <color theme="6" tint="-0.249977111117893"/>
       <name val="Century Gothic"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -790,7 +771,7 @@
     <xf numFmtId="0" fontId="15" fillId="19" borderId="0" applyFont="0"/>
     <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyFont="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -895,57 +876,56 @@
     <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="29" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="16" fillId="16" borderId="2" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="16" fillId="19" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="16" fillId="18" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="16" fillId="16" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="21" fillId="17" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="21" fillId="17" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="19" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="18" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="16" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="16" borderId="2" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Custom Style" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -1742,7 +1722,7 @@
         <v>26</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.45">
@@ -1854,7 +1834,7 @@
         <v>1250</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.45">
@@ -1924,7 +1904,7 @@
         <v>5500</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.45">
@@ -2068,12 +2048,12 @@
       <c r="G1" s="32"/>
     </row>
     <row r="2" spans="2:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="66" t="s">
-        <v>99</v>
-      </c>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
+      <c r="B2" s="60" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
       <c r="F2" s="32"/>
       <c r="G2" s="32"/>
     </row>
@@ -2082,62 +2062,62 @@
         <v>11</v>
       </c>
       <c r="C3" s="33" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="67" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67" t="s">
+        <v>85</v>
+      </c>
+      <c r="G3" s="67"/>
+      <c r="H3" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="I3" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="D3" s="54" t="s">
+      <c r="J3" s="67" t="s">
         <v>88</v>
       </c>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54" t="s">
+      <c r="K3" s="67"/>
+      <c r="L3" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="54"/>
-      <c r="H3" s="34" t="s">
+      <c r="M3" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="I3" s="34" t="s">
+      <c r="N3" s="34" t="s">
         <v>91</v>
-      </c>
-      <c r="J3" s="54" t="s">
-        <v>92</v>
-      </c>
-      <c r="K3" s="54"/>
-      <c r="L3" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="M3" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="N3" s="34" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="4" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="22">
         <f ca="1">NOW()-14</f>
-        <v>45408.645012499997</v>
+        <v>45497.429897916663</v>
       </c>
       <c r="C4" s="23">
         <v>212340</v>
       </c>
-      <c r="D4" s="55" t="s">
-        <v>96</v>
-      </c>
-      <c r="E4" s="55"/>
-      <c r="F4" s="56">
+      <c r="D4" s="68" t="s">
+        <v>92</v>
+      </c>
+      <c r="E4" s="68"/>
+      <c r="F4" s="69">
         <v>250</v>
       </c>
-      <c r="G4" s="56"/>
+      <c r="G4" s="69"/>
       <c r="H4" s="24">
         <v>130</v>
       </c>
       <c r="I4" s="25">
         <v>12.42</v>
       </c>
-      <c r="J4" s="57">
+      <c r="J4" s="70">
         <v>50</v>
       </c>
-      <c r="K4" s="57"/>
+      <c r="K4" s="70"/>
       <c r="L4" s="25">
         <v>8</v>
       </c>
@@ -2152,29 +2132,29 @@
     <row r="5" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B5" s="26">
         <f ca="1">NOW()-13</f>
-        <v>45409.645012499997</v>
+        <v>45498.429897916663</v>
       </c>
       <c r="C5" s="27">
         <v>289043</v>
       </c>
-      <c r="D5" s="58" t="s">
-        <v>96</v>
-      </c>
-      <c r="E5" s="58"/>
-      <c r="F5" s="59">
+      <c r="D5" s="61" t="s">
+        <v>92</v>
+      </c>
+      <c r="E5" s="61"/>
+      <c r="F5" s="62">
         <v>250</v>
       </c>
-      <c r="G5" s="59"/>
+      <c r="G5" s="62"/>
       <c r="H5" s="28">
         <v>0</v>
       </c>
       <c r="I5" s="29">
         <v>26.6</v>
       </c>
-      <c r="J5" s="60">
+      <c r="J5" s="63">
         <v>45</v>
       </c>
-      <c r="K5" s="60"/>
+      <c r="K5" s="63"/>
       <c r="L5" s="29">
         <v>7.8</v>
       </c>
@@ -2189,29 +2169,29 @@
     <row r="6" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="22">
         <f ca="1">NOW()-12</f>
-        <v>45410.645012499997</v>
+        <v>45499.429897916663</v>
       </c>
       <c r="C6" s="23">
         <v>212340</v>
       </c>
-      <c r="D6" s="61" t="s">
-        <v>97</v>
-      </c>
-      <c r="E6" s="61"/>
-      <c r="F6" s="62">
+      <c r="D6" s="64" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" s="64"/>
+      <c r="F6" s="65">
         <v>0</v>
       </c>
-      <c r="G6" s="62"/>
+      <c r="G6" s="65"/>
       <c r="H6" s="24">
         <v>10</v>
       </c>
       <c r="I6" s="25">
         <v>0</v>
       </c>
-      <c r="J6" s="63">
+      <c r="J6" s="66">
         <v>58</v>
       </c>
-      <c r="K6" s="63"/>
+      <c r="K6" s="66"/>
       <c r="L6" s="25">
         <v>2.79</v>
       </c>
@@ -2226,29 +2206,29 @@
     <row r="7" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="26">
         <f ca="1">NOW()-11</f>
-        <v>45411.645012499997</v>
+        <v>45500.429897916663</v>
       </c>
       <c r="C7" s="27">
         <v>216049</v>
       </c>
-      <c r="D7" s="58" t="s">
-        <v>97</v>
-      </c>
-      <c r="E7" s="58"/>
-      <c r="F7" s="59">
+      <c r="D7" s="61" t="s">
+        <v>93</v>
+      </c>
+      <c r="E7" s="61"/>
+      <c r="F7" s="62">
         <v>0</v>
       </c>
-      <c r="G7" s="59"/>
+      <c r="G7" s="62"/>
       <c r="H7" s="28">
         <v>30</v>
       </c>
       <c r="I7" s="29">
         <v>0</v>
       </c>
-      <c r="J7" s="60">
+      <c r="J7" s="63">
         <v>60</v>
       </c>
-      <c r="K7" s="60"/>
+      <c r="K7" s="63"/>
       <c r="L7" s="29">
         <v>9.7899999999999991</v>
       </c>
@@ -2263,29 +2243,29 @@
     <row r="8" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="22">
         <f ca="1">NOW()-10</f>
-        <v>45412.645012499997</v>
+        <v>45501.429897916663</v>
       </c>
       <c r="C8" s="23">
         <v>292352</v>
       </c>
-      <c r="D8" s="61" t="s">
-        <v>96</v>
-      </c>
-      <c r="E8" s="61"/>
-      <c r="F8" s="62">
+      <c r="D8" s="64" t="s">
+        <v>92</v>
+      </c>
+      <c r="E8" s="64"/>
+      <c r="F8" s="65">
         <v>295.5</v>
       </c>
-      <c r="G8" s="62"/>
+      <c r="G8" s="65"/>
       <c r="H8" s="24">
         <v>150</v>
       </c>
       <c r="I8" s="25">
         <v>10.48</v>
       </c>
-      <c r="J8" s="63">
+      <c r="J8" s="66">
         <v>45</v>
       </c>
-      <c r="K8" s="63"/>
+      <c r="K8" s="66"/>
       <c r="L8" s="25">
         <v>9.32</v>
       </c>
@@ -2300,29 +2280,29 @@
     <row r="9" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="26">
         <f ca="1">NOW()-9</f>
-        <v>45413.645012499997</v>
+        <v>45502.429897916663</v>
       </c>
       <c r="C9" s="27">
         <v>567384</v>
       </c>
-      <c r="D9" s="58" t="s">
-        <v>96</v>
-      </c>
-      <c r="E9" s="58"/>
-      <c r="F9" s="59">
+      <c r="D9" s="61" t="s">
+        <v>92</v>
+      </c>
+      <c r="E9" s="61"/>
+      <c r="F9" s="62">
         <v>295.5</v>
       </c>
-      <c r="G9" s="59"/>
+      <c r="G9" s="62"/>
       <c r="H9" s="28">
         <v>30</v>
       </c>
       <c r="I9" s="29">
         <v>20.37</v>
       </c>
-      <c r="J9" s="60">
+      <c r="J9" s="63">
         <v>50</v>
       </c>
-      <c r="K9" s="60"/>
+      <c r="K9" s="63"/>
       <c r="L9" s="29">
         <v>9.1199999999999992</v>
       </c>
@@ -2337,29 +2317,29 @@
     <row r="10" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B10" s="22">
         <f ca="1">NOW()-8</f>
-        <v>45414.645012499997</v>
+        <v>45503.429897916663</v>
       </c>
       <c r="C10" s="23">
         <v>890733</v>
       </c>
-      <c r="D10" s="61" t="s">
-        <v>96</v>
-      </c>
-      <c r="E10" s="61"/>
-      <c r="F10" s="62">
+      <c r="D10" s="64" t="s">
+        <v>92</v>
+      </c>
+      <c r="E10" s="64"/>
+      <c r="F10" s="65">
         <v>349</v>
       </c>
-      <c r="G10" s="62"/>
+      <c r="G10" s="65"/>
       <c r="H10" s="24">
         <v>70</v>
       </c>
       <c r="I10" s="25">
         <v>15.07</v>
       </c>
-      <c r="J10" s="63">
+      <c r="J10" s="66">
         <v>45</v>
       </c>
-      <c r="K10" s="63"/>
+      <c r="K10" s="66"/>
       <c r="L10" s="25">
         <v>14.05</v>
       </c>
@@ -2374,29 +2354,29 @@
     <row r="11" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="26">
         <f ca="1">NOW()-7</f>
-        <v>45415.645012499997</v>
+        <v>45504.429897916663</v>
       </c>
       <c r="C11" s="27">
         <v>578292</v>
       </c>
-      <c r="D11" s="58" t="s">
-        <v>96</v>
-      </c>
-      <c r="E11" s="58"/>
-      <c r="F11" s="59">
+      <c r="D11" s="61" t="s">
+        <v>92</v>
+      </c>
+      <c r="E11" s="61"/>
+      <c r="F11" s="62">
         <v>349</v>
       </c>
-      <c r="G11" s="59"/>
+      <c r="G11" s="62"/>
       <c r="H11" s="28">
         <v>0</v>
       </c>
       <c r="I11" s="29">
         <v>6.8</v>
       </c>
-      <c r="J11" s="60">
+      <c r="J11" s="63">
         <v>60</v>
       </c>
-      <c r="K11" s="60"/>
+      <c r="K11" s="63"/>
       <c r="L11" s="29">
         <v>3.7</v>
       </c>
@@ -2411,29 +2391,29 @@
     <row r="12" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="22">
         <f ca="1">NOW()-6</f>
-        <v>45416.645012499997</v>
+        <v>45505.429897916663</v>
       </c>
       <c r="C12" s="23">
         <v>199123</v>
       </c>
-      <c r="D12" s="61" t="s">
-        <v>96</v>
-      </c>
-      <c r="E12" s="61"/>
-      <c r="F12" s="62">
+      <c r="D12" s="64" t="s">
+        <v>92</v>
+      </c>
+      <c r="E12" s="64"/>
+      <c r="F12" s="65">
         <v>349</v>
       </c>
-      <c r="G12" s="62"/>
+      <c r="G12" s="65"/>
       <c r="H12" s="24">
         <v>90</v>
       </c>
       <c r="I12" s="25">
         <v>13.6</v>
       </c>
-      <c r="J12" s="63">
+      <c r="J12" s="66">
         <v>50</v>
       </c>
-      <c r="K12" s="63"/>
+      <c r="K12" s="66"/>
       <c r="L12" s="25">
         <v>2.6</v>
       </c>
@@ -2448,29 +2428,29 @@
     <row r="13" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B13" s="26">
         <f ca="1">NOW()-5</f>
-        <v>45417.645012499997</v>
+        <v>45506.429897916663</v>
       </c>
       <c r="C13" s="27">
         <v>423509</v>
       </c>
-      <c r="D13" s="58" t="s">
-        <v>97</v>
-      </c>
-      <c r="E13" s="58"/>
-      <c r="F13" s="59">
+      <c r="D13" s="61" t="s">
+        <v>93</v>
+      </c>
+      <c r="E13" s="61"/>
+      <c r="F13" s="62">
         <v>0</v>
       </c>
-      <c r="G13" s="59"/>
+      <c r="G13" s="62"/>
       <c r="H13" s="28">
         <v>0</v>
       </c>
       <c r="I13" s="29">
         <v>37.5</v>
       </c>
-      <c r="J13" s="60">
+      <c r="J13" s="63">
         <v>60</v>
       </c>
-      <c r="K13" s="60"/>
+      <c r="K13" s="63"/>
       <c r="L13" s="29">
         <v>2.04</v>
       </c>
@@ -2485,29 +2465,29 @@
     <row r="14" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B14" s="22">
         <f ca="1">NOW()-4</f>
-        <v>45418.645012499997</v>
+        <v>45507.429897916663</v>
       </c>
       <c r="C14" s="23">
         <v>543288</v>
       </c>
-      <c r="D14" s="61" t="s">
-        <v>97</v>
-      </c>
-      <c r="E14" s="61"/>
-      <c r="F14" s="62">
+      <c r="D14" s="64" t="s">
+        <v>93</v>
+      </c>
+      <c r="E14" s="64"/>
+      <c r="F14" s="65">
         <v>0</v>
       </c>
-      <c r="G14" s="62"/>
+      <c r="G14" s="65"/>
       <c r="H14" s="24">
         <v>90</v>
       </c>
       <c r="I14" s="25">
         <v>14.2</v>
       </c>
-      <c r="J14" s="63">
+      <c r="J14" s="66">
         <v>70</v>
       </c>
-      <c r="K14" s="63"/>
+      <c r="K14" s="66"/>
       <c r="L14" s="25">
         <v>0.2</v>
       </c>
@@ -2522,29 +2502,29 @@
     <row r="15" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B15" s="26">
         <f ca="1">NOW()-3</f>
-        <v>45419.645012499997</v>
+        <v>45508.429897916663</v>
       </c>
       <c r="C15" s="27">
         <v>457382</v>
       </c>
-      <c r="D15" s="58" t="s">
-        <v>96</v>
-      </c>
-      <c r="E15" s="58"/>
-      <c r="F15" s="59">
+      <c r="D15" s="61" t="s">
+        <v>92</v>
+      </c>
+      <c r="E15" s="61"/>
+      <c r="F15" s="62">
         <v>205</v>
       </c>
-      <c r="G15" s="59"/>
+      <c r="G15" s="62"/>
       <c r="H15" s="28">
         <v>125</v>
       </c>
       <c r="I15" s="29">
         <v>16</v>
       </c>
-      <c r="J15" s="60">
+      <c r="J15" s="63">
         <v>45</v>
       </c>
-      <c r="K15" s="60"/>
+      <c r="K15" s="63"/>
       <c r="L15" s="29">
         <v>14</v>
       </c>
@@ -2559,29 +2539,29 @@
     <row r="16" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B16" s="22">
         <f ca="1">NOW()-2</f>
-        <v>45420.645012499997</v>
+        <v>45509.429897916663</v>
       </c>
       <c r="C16" s="23">
         <v>584839</v>
       </c>
-      <c r="D16" s="61" t="s">
-        <v>96</v>
-      </c>
-      <c r="E16" s="61"/>
-      <c r="F16" s="62">
+      <c r="D16" s="64" t="s">
+        <v>92</v>
+      </c>
+      <c r="E16" s="64"/>
+      <c r="F16" s="65">
         <v>205</v>
       </c>
-      <c r="G16" s="62"/>
+      <c r="G16" s="65"/>
       <c r="H16" s="24">
         <v>0</v>
       </c>
       <c r="I16" s="25">
         <v>10.029999999999999</v>
       </c>
-      <c r="J16" s="63">
+      <c r="J16" s="66">
         <v>40</v>
       </c>
-      <c r="K16" s="63"/>
+      <c r="K16" s="66"/>
       <c r="L16" s="25">
         <v>12.01</v>
       </c>
@@ -2596,29 +2576,29 @@
     <row r="17" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B17" s="26">
         <f ca="1">NOW()-1</f>
-        <v>45421.645012499997</v>
+        <v>45510.429897916663</v>
       </c>
       <c r="C17" s="27">
         <v>483922</v>
       </c>
-      <c r="D17" s="58" t="s">
-        <v>96</v>
-      </c>
-      <c r="E17" s="58"/>
-      <c r="F17" s="59">
+      <c r="D17" s="61" t="s">
+        <v>92</v>
+      </c>
+      <c r="E17" s="61"/>
+      <c r="F17" s="62">
         <v>205</v>
       </c>
-      <c r="G17" s="59"/>
+      <c r="G17" s="62"/>
       <c r="H17" s="28">
         <v>0</v>
       </c>
       <c r="I17" s="29">
         <v>26</v>
       </c>
-      <c r="J17" s="60">
+      <c r="J17" s="63">
         <v>55</v>
       </c>
-      <c r="K17" s="60"/>
+      <c r="K17" s="63"/>
       <c r="L17" s="29">
         <v>9.1999999999999993</v>
       </c>
@@ -2633,29 +2613,29 @@
     <row r="18" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B18" s="22">
         <f ca="1">NOW()</f>
-        <v>45422.645012499997</v>
+        <v>45511.429897916663</v>
       </c>
       <c r="C18" s="23">
         <v>890763</v>
       </c>
-      <c r="D18" s="61" t="s">
-        <v>96</v>
-      </c>
-      <c r="E18" s="61"/>
-      <c r="F18" s="62">
+      <c r="D18" s="64" t="s">
+        <v>92</v>
+      </c>
+      <c r="E18" s="64"/>
+      <c r="F18" s="65">
         <v>205</v>
       </c>
-      <c r="G18" s="62"/>
+      <c r="G18" s="65"/>
       <c r="H18" s="24">
         <v>125</v>
       </c>
       <c r="I18" s="25">
         <v>9.5</v>
       </c>
-      <c r="J18" s="63">
+      <c r="J18" s="66">
         <v>45</v>
       </c>
-      <c r="K18" s="63"/>
+      <c r="K18" s="66"/>
       <c r="L18" s="25">
         <v>1.03</v>
       </c>
@@ -2670,13 +2650,13 @@
     <row r="19" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B19" s="30"/>
       <c r="C19" s="30"/>
-      <c r="D19" s="64"/>
-      <c r="E19" s="64"/>
-      <c r="F19" s="65">
+      <c r="D19" s="58"/>
+      <c r="E19" s="58"/>
+      <c r="F19" s="59">
         <f>SUM(F4:G18)</f>
         <v>2958</v>
       </c>
-      <c r="G19" s="65"/>
+      <c r="G19" s="59"/>
       <c r="H19" s="36">
         <f t="shared" ref="H19:I19" si="1">SUM(H3:H18)</f>
         <v>850</v>
@@ -2685,11 +2665,11 @@
         <f t="shared" si="1"/>
         <v>218.56999999999996</v>
       </c>
-      <c r="J19" s="65">
+      <c r="J19" s="59">
         <f>SUM(J4:K18)</f>
         <v>778</v>
       </c>
-      <c r="K19" s="65"/>
+      <c r="K19" s="59"/>
       <c r="L19" s="36">
         <f t="shared" ref="L19:M19" si="2">SUM(L4:L18)</f>
         <v>105.65000000000002</v>
@@ -2713,7 +2693,7 @@
       <c r="K20" s="30"/>
       <c r="L20" s="30"/>
       <c r="M20" s="40" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="N20" s="37">
         <f>SUM(N4:N18)</f>
@@ -2722,6 +2702,42 @@
     </row>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="J14:K14"/>
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="F19:G19"/>
     <mergeCell ref="J19:K19"/>
@@ -2738,42 +2754,6 @@
     <mergeCell ref="D16:E16"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="J16:K16"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="J4:K4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
@@ -2789,48 +2769,48 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B3" s="67"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
+      <c r="B3" s="71"/>
+      <c r="C3" s="71"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B4" s="67"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="67"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="67"/>
-      <c r="G4" s="67"/>
-      <c r="H4" s="67"/>
-      <c r="I4" s="67"/>
-      <c r="J4" s="67"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="71"/>
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
+      <c r="F4" s="71"/>
+      <c r="G4" s="71"/>
+      <c r="H4" s="71"/>
+      <c r="I4" s="71"/>
+      <c r="J4" s="71"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B5" s="67"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
-      <c r="H5" s="67"/>
-      <c r="I5" s="67"/>
-      <c r="J5" s="67"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="71"/>
+      <c r="D5" s="71"/>
+      <c r="E5" s="71"/>
+      <c r="F5" s="71"/>
+      <c r="G5" s="71"/>
+      <c r="H5" s="71"/>
+      <c r="I5" s="71"/>
+      <c r="J5" s="71"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3132,13 +3112,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B1" s="68" t="s">
+      <c r="B1" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B3" s="2" t="s">
@@ -3224,13 +3204,13 @@
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B10" s="68" t="s">
+      <c r="B10" s="72" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="68"/>
+      <c r="C10" s="72"/>
+      <c r="D10" s="72"/>
+      <c r="E10" s="72"/>
+      <c r="F10" s="72"/>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B12" s="2" t="s">
@@ -3334,27 +3314,23 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="16.1328125" customWidth="1"/>
     <col min="2" max="2" width="25.59765625" customWidth="1"/>
-    <col min="4" max="4" width="20.3984375" customWidth="1"/>
-    <col min="5" max="5" width="15.1328125" customWidth="1"/>
-    <col min="6" max="6" width="22.265625" customWidth="1"/>
+    <col min="4" max="4" width="22.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="69" t="s">
+    <row r="1" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="73" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" s="16" t="s">
         <v>34</v>
       </c>
@@ -3367,416 +3343,276 @@
       <c r="D2" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="16" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A3" s="43" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="54">
+        <v>997061</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A4" s="43" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" s="54">
+        <v>962909</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A5" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="54">
+        <v>956207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A6" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="B6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="54">
+        <v>854740</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="54">
+        <v>774122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A8" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="55">
+        <v>328726</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A9" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A3" s="45" t="s">
+      <c r="C9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="55">
+        <v>278040</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A10" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="55">
+        <v>214969</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A11" s="43" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="55">
+        <v>195820</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A12" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="55">
+        <v>190457</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A13" s="46" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" s="55">
+        <v>122104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A14" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" s="56">
+        <v>77482</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A15" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D3">
-        <v>142958</v>
-      </c>
-      <c r="E3">
-        <v>1524915</v>
-      </c>
-      <c r="F3" s="70">
-        <v>1707540</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A4" s="43" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="D15" s="56">
+        <v>55150</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A16" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="56">
+        <v>50599</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A17" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D4">
-        <v>34017</v>
-      </c>
-      <c r="E4">
-        <v>1577040</v>
-      </c>
-      <c r="F4" s="71">
-        <v>997061</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A5" s="43" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" t="s">
-        <v>83</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D5">
-        <v>310384</v>
-      </c>
-      <c r="E5">
-        <v>14419400</v>
-      </c>
-      <c r="F5" s="71">
-        <v>962909</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A6" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="B17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="56">
+        <v>37780</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A18" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6">
-        <v>1348932</v>
-      </c>
-      <c r="E6">
-        <v>5949786</v>
-      </c>
-      <c r="F6" s="71">
-        <v>956207</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A7" s="41" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D7">
-        <v>194946</v>
-      </c>
-      <c r="E7">
-        <v>2143035</v>
-      </c>
-      <c r="F7" s="71">
-        <v>854740</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A8" s="42" t="s">
-        <v>43</v>
-      </c>
-      <c r="B8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8">
-        <v>22268</v>
-      </c>
-      <c r="E8">
-        <v>1138262</v>
-      </c>
-      <c r="F8" s="71">
-        <v>774122</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A9" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9">
-        <v>1224614</v>
-      </c>
-      <c r="E9">
-        <v>1710917</v>
-      </c>
-      <c r="F9" s="72">
-        <v>328726</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A10" s="41" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10">
-        <v>40412</v>
-      </c>
-      <c r="E10">
-        <v>368736</v>
-      </c>
-      <c r="F10" s="72">
-        <v>278040</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A11" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="B11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="B18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="56">
+        <v>35703</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A19" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" s="56">
+        <v>30134</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A20" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="57">
+        <v>24291</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A21" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" t="s">
         <v>71</v>
       </c>
-      <c r="D11">
-        <v>27448</v>
-      </c>
-      <c r="E11">
-        <v>526811</v>
-      </c>
-      <c r="F11" s="72">
-        <v>214969</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A12" s="43" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D12">
-        <v>113423</v>
-      </c>
-      <c r="E12">
-        <v>1034941</v>
-      </c>
-      <c r="F12" s="72">
-        <v>195820</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A13" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="B13" t="s">
-        <v>60</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13">
-        <v>239871</v>
-      </c>
-      <c r="E13">
-        <v>709266</v>
-      </c>
-      <c r="F13" s="72">
-        <v>190457</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A14" s="46" t="s">
+      <c r="C21" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B14" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14">
-        <v>50133</v>
-      </c>
-      <c r="E14">
-        <v>363241</v>
-      </c>
-      <c r="F14" s="72">
-        <v>122104</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A15" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="B15" t="s">
-        <v>79</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D15">
-        <v>72752</v>
-      </c>
-      <c r="E15">
-        <v>731144</v>
-      </c>
-      <c r="F15" s="73">
-        <v>77482</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A16" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" t="s">
-        <v>54</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D16">
-        <v>62787</v>
-      </c>
-      <c r="E16">
-        <v>2548315</v>
-      </c>
-      <c r="F16" s="73">
-        <v>55150</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A17" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" t="s">
-        <v>77</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D17">
-        <v>46077</v>
-      </c>
-      <c r="E17">
-        <v>1380109</v>
-      </c>
-      <c r="F17" s="73">
-        <v>50599</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A18" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="B18" t="s">
-        <v>64</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D18">
-        <v>126536</v>
-      </c>
-      <c r="E18">
-        <v>5495379</v>
-      </c>
-      <c r="F18" s="73">
-        <v>37780</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A19" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="B19" t="s">
-        <v>56</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D19">
-        <v>82302</v>
-      </c>
-      <c r="E19">
-        <v>3284474</v>
-      </c>
-      <c r="F19" s="73">
-        <v>35703</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A20" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D20">
-        <v>60551</v>
-      </c>
-      <c r="E20">
-        <v>2041955</v>
-      </c>
-      <c r="F20" s="73">
-        <v>30134</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A21" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" t="s">
-        <v>81</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D21">
-        <v>62036</v>
-      </c>
-      <c r="E21">
-        <v>2548315</v>
-      </c>
-      <c r="F21" s="74">
-        <v>24291</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A22" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="B22" t="s">
-        <v>75</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D22">
-        <v>48184</v>
-      </c>
-      <c r="E22">
-        <v>1014890</v>
-      </c>
-      <c r="F22" s="74">
+      <c r="D21" s="57">
         <v>9926</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" fitToHeight="0" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>

</xml_diff>